<commit_message>
Add a Priority field to master requirements, top to bottom
Adds an admin-settable High/Medium/Low priority to master requirements:
a new column in the Master Requirement import template and workbook
parser (validated, with a same-ID consistency check like requirement
text), a Priority select in the requirement editor, a compact column
in the import review grid, and a priority pill on the import batch
preview.

While rebuilding the import templates to add the column, discovered
both .xlsx files' internal zip entries used backslash path separators
instead of the OOXML-required forward slashes — SheetJS tolerates it,
but stricter readers (ExcelJS, likely others) silently see zero
sheets. Repacked both templates with correct paths; content is
otherwise unchanged for Site-Import-Template.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/Site-Import-Template.xlsx
+++ b/public/templates/Site-Import-Template.xlsx
@@ -1,29 +1,22 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>Microsoft Excel</Application>
-  <TitlesOfParts>
-    <vt:vector size="4" baseType="lpstr">
-      <vt:lpstr>Instructions</vt:lpstr>
-      <vt:lpstr>Import Template</vt:lpstr>
-      <vt:lpstr>Sample Data</vt:lpstr>
-      <vt:lpstr>Lookup Lists</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14000" firstSheet="1" activeTab="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
+    <sheet name="Import Template" sheetId="2" r:id="rId2"/>
+    <sheet name="Sample Data" sheetId="3" r:id="rId3"/>
+    <sheet name="Lookup Lists" sheetId="4" r:id="rId4"/>
+  </sheets>
+  <calcPr calcId="191028"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:title>EHS360 Site Import Template</dc:title>
-  <dc:creator>Maitsys Assure</dc:creator>
-  <cp:lastModifiedBy>Maitsys Assure</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-01-01T00:00:00Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-01-01T00:00:00Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t xml:space="preserve">EHS360 - Site Import Template</t>
@@ -250,7 +243,7 @@
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11">
     <font>
@@ -432,7 +425,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -715,24 +708,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14000" firstSheet="1" activeTab="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Instructions" sheetId="1" r:id="rId1"/>
-    <sheet name="Import Template" sheetId="2" r:id="rId2"/>
-    <sheet name="Sample Data" sheetId="3" r:id="rId3"/>
-    <sheet name="Lookup Lists" sheetId="4" r:id="rId4"/>
-  </sheets>
-  <calcPr calcId="191028"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -928,7 +904,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr">
   <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1250,7 +1226,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr">
   <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1456,7 +1432,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>